<commit_message>
stage(4): confirm final results + tag stage4-results
Q1 子问 1 (waste) = 1106.79 万元
Q1 子问 2 (discount) = 940.05 万元
Q2 (n=500, sigma=0.10) = 953.84 ± 354.40 万元, CV=0.37
Q3 (n=300, elastic+legume) = 1224.01 万元, CV=0.30, vs Q2 +28.3%

- main.tex 摘要与结果表填入实际数字
- writer.md 阶段 4 状态更新, 写入已知限制
- outputs/result_summary.xlsx + result_summary.csv 汇总三问 + 约束校验
- 重新生成 figures/q2_robust_path.png 等

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2024C/outputs/result2.xlsx
+++ b/2024C/outputs/result2.xlsx
@@ -1367,9 +1367,6 @@
           <t>D1</t>
         </is>
       </c>
-      <c r="AK55" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1397,9 +1394,6 @@
           <t>D2</t>
         </is>
       </c>
-      <c r="AK57" t="n">
-        <v>10</v>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1427,9 +1421,6 @@
           <t>D3</t>
         </is>
       </c>
-      <c r="AK59" t="n">
-        <v>14</v>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1457,9 +1448,6 @@
           <t>D4</t>
         </is>
       </c>
-      <c r="AK61" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1487,9 +1475,6 @@
           <t>D5</t>
         </is>
       </c>
-      <c r="AK63" t="n">
-        <v>10</v>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1517,9 +1502,6 @@
           <t>D6</t>
         </is>
       </c>
-      <c r="AK65" t="n">
-        <v>12</v>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1547,9 +1529,6 @@
           <t>D7</t>
         </is>
       </c>
-      <c r="AK67" t="n">
-        <v>22</v>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1577,9 +1556,6 @@
           <t>D8</t>
         </is>
       </c>
-      <c r="AK69" t="n">
-        <v>20</v>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1592,9 +1568,6 @@
           <t>E1</t>
         </is>
       </c>
-      <c r="AE70" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1622,9 +1595,6 @@
           <t>E2</t>
         </is>
       </c>
-      <c r="AE72" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1652,9 +1622,6 @@
           <t>E3</t>
         </is>
       </c>
-      <c r="AE74" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1682,9 +1649,6 @@
           <t>E4</t>
         </is>
       </c>
-      <c r="AE76" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1712,9 +1676,6 @@
           <t>E5</t>
         </is>
       </c>
-      <c r="AE78" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1742,9 +1703,6 @@
           <t>E6</t>
         </is>
       </c>
-      <c r="AE80" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1772,9 +1730,6 @@
           <t>E7</t>
         </is>
       </c>
-      <c r="AE82" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1802,9 +1757,6 @@
           <t>E8</t>
         </is>
       </c>
-      <c r="AE84" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1832,9 +1784,6 @@
           <t>E9</t>
         </is>
       </c>
-      <c r="AE86" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1862,9 +1811,6 @@
           <t>E10</t>
         </is>
       </c>
-      <c r="AE88" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1892,9 +1838,6 @@
           <t>E11</t>
         </is>
       </c>
-      <c r="AE90" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1922,9 +1865,6 @@
           <t>E12</t>
         </is>
       </c>
-      <c r="AE92" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1952,9 +1892,6 @@
           <t>E13</t>
         </is>
       </c>
-      <c r="AE94" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1982,9 +1919,6 @@
           <t>E14</t>
         </is>
       </c>
-      <c r="AE96" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2012,9 +1946,6 @@
           <t>E15</t>
         </is>
       </c>
-      <c r="AE98" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2042,9 +1973,6 @@
           <t>E16</t>
         </is>
       </c>
-      <c r="AE100" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2072,9 +2000,6 @@
           <t>F1</t>
         </is>
       </c>
-      <c r="AH102" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2102,9 +2027,6 @@
           <t>F2</t>
         </is>
       </c>
-      <c r="AH104" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -2132,9 +2054,6 @@
           <t>F3</t>
         </is>
       </c>
-      <c r="AH106" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2161,9 +2080,6 @@
         <is>
           <t>F4</t>
         </is>
-      </c>
-      <c r="AH108" t="n">
-        <v>0.6</v>
       </c>
     </row>
     <row r="109">
@@ -3140,9 +3056,6 @@
           <t>D1</t>
         </is>
       </c>
-      <c r="AL55" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3170,9 +3083,6 @@
           <t>D2</t>
         </is>
       </c>
-      <c r="AL57" t="n">
-        <v>10</v>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3200,9 +3110,6 @@
           <t>D3</t>
         </is>
       </c>
-      <c r="AL59" t="n">
-        <v>14</v>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3230,9 +3137,6 @@
           <t>D4</t>
         </is>
       </c>
-      <c r="AL61" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3260,9 +3164,6 @@
           <t>D5</t>
         </is>
       </c>
-      <c r="AL63" t="n">
-        <v>10</v>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3290,9 +3191,6 @@
           <t>D6</t>
         </is>
       </c>
-      <c r="AL65" t="n">
-        <v>12</v>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3320,9 +3218,6 @@
           <t>D7</t>
         </is>
       </c>
-      <c r="AL67" t="n">
-        <v>22</v>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3350,9 +3245,6 @@
           <t>D8</t>
         </is>
       </c>
-      <c r="AL69" t="n">
-        <v>20</v>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3365,9 +3257,6 @@
           <t>E1</t>
         </is>
       </c>
-      <c r="AH70" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3395,9 +3284,6 @@
           <t>E2</t>
         </is>
       </c>
-      <c r="AH72" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3425,9 +3311,6 @@
           <t>E3</t>
         </is>
       </c>
-      <c r="AH74" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3455,9 +3338,6 @@
           <t>E4</t>
         </is>
       </c>
-      <c r="AH76" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3485,9 +3365,6 @@
           <t>E5</t>
         </is>
       </c>
-      <c r="AH78" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3515,9 +3392,6 @@
           <t>E6</t>
         </is>
       </c>
-      <c r="AH80" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3545,9 +3419,6 @@
           <t>E7</t>
         </is>
       </c>
-      <c r="AH82" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3575,9 +3446,6 @@
           <t>E8</t>
         </is>
       </c>
-      <c r="AH84" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3605,9 +3473,6 @@
           <t>E9</t>
         </is>
       </c>
-      <c r="AH86" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3635,9 +3500,6 @@
           <t>E10</t>
         </is>
       </c>
-      <c r="AH88" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3665,9 +3527,6 @@
           <t>E11</t>
         </is>
       </c>
-      <c r="AH90" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3695,9 +3554,6 @@
           <t>E12</t>
         </is>
       </c>
-      <c r="AH92" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3725,9 +3581,6 @@
           <t>E13</t>
         </is>
       </c>
-      <c r="AH94" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3755,9 +3608,6 @@
           <t>E14</t>
         </is>
       </c>
-      <c r="AH96" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3785,9 +3635,6 @@
           <t>E15</t>
         </is>
       </c>
-      <c r="AH98" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3815,9 +3662,6 @@
           <t>E16</t>
         </is>
       </c>
-      <c r="AH100" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3860,9 +3704,6 @@
           <t>F1</t>
         </is>
       </c>
-      <c r="AH103" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -3890,9 +3731,6 @@
           <t>F2</t>
         </is>
       </c>
-      <c r="AH105" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -3920,9 +3758,6 @@
           <t>F3</t>
         </is>
       </c>
-      <c r="AH107" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3949,9 +3784,6 @@
         <is>
           <t>F4</t>
         </is>
-      </c>
-      <c r="AH109" t="n">
-        <v>0.6</v>
       </c>
     </row>
   </sheetData>
@@ -4913,9 +4745,6 @@
           <t>D1</t>
         </is>
       </c>
-      <c r="AK55" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4943,9 +4772,6 @@
           <t>D2</t>
         </is>
       </c>
-      <c r="AK57" t="n">
-        <v>10</v>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4973,9 +4799,6 @@
           <t>D3</t>
         </is>
       </c>
-      <c r="AK59" t="n">
-        <v>14</v>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5003,9 +4826,6 @@
           <t>D4</t>
         </is>
       </c>
-      <c r="AK61" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5033,9 +4853,6 @@
           <t>D5</t>
         </is>
       </c>
-      <c r="AK63" t="n">
-        <v>10</v>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5063,9 +4880,6 @@
           <t>D6</t>
         </is>
       </c>
-      <c r="AK65" t="n">
-        <v>12</v>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5093,9 +4907,6 @@
           <t>D7</t>
         </is>
       </c>
-      <c r="AK67" t="n">
-        <v>22</v>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5123,9 +4934,6 @@
           <t>D8</t>
         </is>
       </c>
-      <c r="AK69" t="n">
-        <v>20</v>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5138,9 +4946,6 @@
           <t>E1</t>
         </is>
       </c>
-      <c r="AE70" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5168,9 +4973,6 @@
           <t>E2</t>
         </is>
       </c>
-      <c r="AE72" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5198,9 +5000,6 @@
           <t>E3</t>
         </is>
       </c>
-      <c r="AE74" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5228,9 +5027,6 @@
           <t>E4</t>
         </is>
       </c>
-      <c r="AE76" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5258,9 +5054,6 @@
           <t>E5</t>
         </is>
       </c>
-      <c r="AE78" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -5288,9 +5081,6 @@
           <t>E6</t>
         </is>
       </c>
-      <c r="AE80" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5318,9 +5108,6 @@
           <t>E7</t>
         </is>
       </c>
-      <c r="AE82" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -5348,9 +5135,6 @@
           <t>E8</t>
         </is>
       </c>
-      <c r="AE84" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -5378,9 +5162,6 @@
           <t>E9</t>
         </is>
       </c>
-      <c r="AE86" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -5408,9 +5189,6 @@
           <t>E10</t>
         </is>
       </c>
-      <c r="AE88" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -5438,9 +5216,6 @@
           <t>E11</t>
         </is>
       </c>
-      <c r="AE90" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5468,9 +5243,6 @@
           <t>E12</t>
         </is>
       </c>
-      <c r="AE92" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5498,9 +5270,6 @@
           <t>E13</t>
         </is>
       </c>
-      <c r="AE94" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5528,9 +5297,6 @@
           <t>E14</t>
         </is>
       </c>
-      <c r="AE96" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5558,9 +5324,6 @@
           <t>E15</t>
         </is>
       </c>
-      <c r="AE98" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5588,9 +5351,6 @@
           <t>E16</t>
         </is>
       </c>
-      <c r="AE100" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5618,9 +5378,6 @@
           <t>F1</t>
         </is>
       </c>
-      <c r="AH102" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -5648,9 +5405,6 @@
           <t>F2</t>
         </is>
       </c>
-      <c r="AH104" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -5678,9 +5432,6 @@
           <t>F3</t>
         </is>
       </c>
-      <c r="AH106" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -5707,9 +5458,6 @@
         <is>
           <t>F4</t>
         </is>
-      </c>
-      <c r="AH108" t="n">
-        <v>0.6</v>
       </c>
     </row>
     <row r="109">
@@ -6686,9 +6434,6 @@
           <t>D1</t>
         </is>
       </c>
-      <c r="AL55" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -6716,9 +6461,6 @@
           <t>D2</t>
         </is>
       </c>
-      <c r="AL57" t="n">
-        <v>10</v>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -6746,9 +6488,6 @@
           <t>D3</t>
         </is>
       </c>
-      <c r="AL59" t="n">
-        <v>14</v>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6776,9 +6515,6 @@
           <t>D4</t>
         </is>
       </c>
-      <c r="AL61" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -6806,9 +6542,6 @@
           <t>D5</t>
         </is>
       </c>
-      <c r="AL63" t="n">
-        <v>10</v>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -6836,9 +6569,6 @@
           <t>D6</t>
         </is>
       </c>
-      <c r="AL65" t="n">
-        <v>12</v>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -6866,9 +6596,6 @@
           <t>D7</t>
         </is>
       </c>
-      <c r="AL67" t="n">
-        <v>22</v>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -6896,9 +6623,6 @@
           <t>D8</t>
         </is>
       </c>
-      <c r="AL69" t="n">
-        <v>20</v>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -6911,9 +6635,6 @@
           <t>E1</t>
         </is>
       </c>
-      <c r="AH70" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -6941,9 +6662,6 @@
           <t>E2</t>
         </is>
       </c>
-      <c r="AH72" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -6971,9 +6689,6 @@
           <t>E3</t>
         </is>
       </c>
-      <c r="AH74" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -7001,9 +6716,6 @@
           <t>E4</t>
         </is>
       </c>
-      <c r="AH76" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -7031,9 +6743,6 @@
           <t>E5</t>
         </is>
       </c>
-      <c r="AH78" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -7061,9 +6770,6 @@
           <t>E6</t>
         </is>
       </c>
-      <c r="AH80" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -7091,9 +6797,6 @@
           <t>E7</t>
         </is>
       </c>
-      <c r="AH82" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -7121,9 +6824,6 @@
           <t>E8</t>
         </is>
       </c>
-      <c r="AH84" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -7151,9 +6851,6 @@
           <t>E9</t>
         </is>
       </c>
-      <c r="AH86" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -7181,9 +6878,6 @@
           <t>E10</t>
         </is>
       </c>
-      <c r="AH88" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -7211,9 +6905,6 @@
           <t>E11</t>
         </is>
       </c>
-      <c r="AH90" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -7241,9 +6932,6 @@
           <t>E12</t>
         </is>
       </c>
-      <c r="AH92" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -7271,9 +6959,6 @@
           <t>E13</t>
         </is>
       </c>
-      <c r="AH94" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -7301,9 +6986,6 @@
           <t>E14</t>
         </is>
       </c>
-      <c r="AH96" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -7331,9 +7013,6 @@
           <t>E15</t>
         </is>
       </c>
-      <c r="AH98" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -7361,9 +7040,6 @@
           <t>E16</t>
         </is>
       </c>
-      <c r="AH100" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -7406,9 +7082,6 @@
           <t>F1</t>
         </is>
       </c>
-      <c r="AH103" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -7436,9 +7109,6 @@
           <t>F2</t>
         </is>
       </c>
-      <c r="AH105" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -7466,9 +7136,6 @@
           <t>F3</t>
         </is>
       </c>
-      <c r="AH107" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -7495,9 +7162,6 @@
         <is>
           <t>F4</t>
         </is>
-      </c>
-      <c r="AH109" t="n">
-        <v>0.6</v>
       </c>
     </row>
   </sheetData>
@@ -8459,9 +8123,6 @@
           <t>D1</t>
         </is>
       </c>
-      <c r="AK55" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -8489,9 +8150,6 @@
           <t>D2</t>
         </is>
       </c>
-      <c r="AK57" t="n">
-        <v>10</v>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -8519,9 +8177,6 @@
           <t>D3</t>
         </is>
       </c>
-      <c r="AK59" t="n">
-        <v>14</v>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -8549,9 +8204,6 @@
           <t>D4</t>
         </is>
       </c>
-      <c r="AK61" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -8579,9 +8231,6 @@
           <t>D5</t>
         </is>
       </c>
-      <c r="AK63" t="n">
-        <v>10</v>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -8609,9 +8258,6 @@
           <t>D6</t>
         </is>
       </c>
-      <c r="AK65" t="n">
-        <v>12</v>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -8639,9 +8285,6 @@
           <t>D7</t>
         </is>
       </c>
-      <c r="AK67" t="n">
-        <v>22</v>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -8669,9 +8312,6 @@
           <t>D8</t>
         </is>
       </c>
-      <c r="AK69" t="n">
-        <v>20</v>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -8684,9 +8324,6 @@
           <t>E1</t>
         </is>
       </c>
-      <c r="AE70" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -8714,9 +8351,6 @@
           <t>E2</t>
         </is>
       </c>
-      <c r="AE72" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -8744,9 +8378,6 @@
           <t>E3</t>
         </is>
       </c>
-      <c r="AE74" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -8774,9 +8405,6 @@
           <t>E4</t>
         </is>
       </c>
-      <c r="AE76" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -8804,9 +8432,6 @@
           <t>E5</t>
         </is>
       </c>
-      <c r="AE78" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -8834,9 +8459,6 @@
           <t>E6</t>
         </is>
       </c>
-      <c r="AE80" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -8864,9 +8486,6 @@
           <t>E7</t>
         </is>
       </c>
-      <c r="AE82" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -8894,9 +8513,6 @@
           <t>E8</t>
         </is>
       </c>
-      <c r="AE84" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -8924,9 +8540,6 @@
           <t>E9</t>
         </is>
       </c>
-      <c r="AE86" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -8954,9 +8567,6 @@
           <t>E10</t>
         </is>
       </c>
-      <c r="AE88" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -8984,9 +8594,6 @@
           <t>E11</t>
         </is>
       </c>
-      <c r="AE90" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -9014,9 +8621,6 @@
           <t>E12</t>
         </is>
       </c>
-      <c r="AE92" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -9044,9 +8648,6 @@
           <t>E13</t>
         </is>
       </c>
-      <c r="AE94" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -9074,9 +8675,6 @@
           <t>E14</t>
         </is>
       </c>
-      <c r="AE96" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -9104,9 +8702,6 @@
           <t>E15</t>
         </is>
       </c>
-      <c r="AE98" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -9134,9 +8729,6 @@
           <t>E16</t>
         </is>
       </c>
-      <c r="AE100" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -9164,9 +8756,6 @@
           <t>F1</t>
         </is>
       </c>
-      <c r="AH102" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -9194,9 +8783,6 @@
           <t>F2</t>
         </is>
       </c>
-      <c r="AH104" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -9224,9 +8810,6 @@
           <t>F3</t>
         </is>
       </c>
-      <c r="AH106" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -9253,9 +8836,6 @@
         <is>
           <t>F4</t>
         </is>
-      </c>
-      <c r="AH108" t="n">
-        <v>0.6</v>
       </c>
     </row>
     <row r="109">
@@ -10232,9 +9812,6 @@
           <t>D1</t>
         </is>
       </c>
-      <c r="AL55" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -10262,9 +9839,6 @@
           <t>D2</t>
         </is>
       </c>
-      <c r="AL57" t="n">
-        <v>10</v>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -10292,9 +9866,6 @@
           <t>D3</t>
         </is>
       </c>
-      <c r="AL59" t="n">
-        <v>14</v>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -10322,9 +9893,6 @@
           <t>D4</t>
         </is>
       </c>
-      <c r="AL61" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -10352,9 +9920,6 @@
           <t>D5</t>
         </is>
       </c>
-      <c r="AL63" t="n">
-        <v>10</v>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -10382,9 +9947,6 @@
           <t>D6</t>
         </is>
       </c>
-      <c r="AL65" t="n">
-        <v>12</v>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -10412,9 +9974,6 @@
           <t>D7</t>
         </is>
       </c>
-      <c r="AL67" t="n">
-        <v>22</v>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -10442,9 +10001,6 @@
           <t>D8</t>
         </is>
       </c>
-      <c r="AL69" t="n">
-        <v>20</v>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -10457,9 +10013,6 @@
           <t>E1</t>
         </is>
       </c>
-      <c r="AH70" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -10487,9 +10040,6 @@
           <t>E2</t>
         </is>
       </c>
-      <c r="AH72" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -10517,9 +10067,6 @@
           <t>E3</t>
         </is>
       </c>
-      <c r="AH74" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -10547,9 +10094,6 @@
           <t>E4</t>
         </is>
       </c>
-      <c r="AH76" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -10577,9 +10121,6 @@
           <t>E5</t>
         </is>
       </c>
-      <c r="AH78" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -10607,9 +10148,6 @@
           <t>E6</t>
         </is>
       </c>
-      <c r="AH80" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -10637,9 +10175,6 @@
           <t>E7</t>
         </is>
       </c>
-      <c r="AH82" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -10667,9 +10202,6 @@
           <t>E8</t>
         </is>
       </c>
-      <c r="AH84" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -10697,9 +10229,6 @@
           <t>E9</t>
         </is>
       </c>
-      <c r="AH86" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -10727,9 +10256,6 @@
           <t>E10</t>
         </is>
       </c>
-      <c r="AH88" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -10757,9 +10283,6 @@
           <t>E11</t>
         </is>
       </c>
-      <c r="AH90" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -10787,9 +10310,6 @@
           <t>E12</t>
         </is>
       </c>
-      <c r="AH92" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -10817,9 +10337,6 @@
           <t>E13</t>
         </is>
       </c>
-      <c r="AH94" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -10847,9 +10364,6 @@
           <t>E14</t>
         </is>
       </c>
-      <c r="AH96" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -10877,9 +10391,6 @@
           <t>E15</t>
         </is>
       </c>
-      <c r="AH98" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -10907,9 +10418,6 @@
           <t>E16</t>
         </is>
       </c>
-      <c r="AH100" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -10952,9 +10460,6 @@
           <t>F1</t>
         </is>
       </c>
-      <c r="AH103" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -10982,9 +10487,6 @@
           <t>F2</t>
         </is>
       </c>
-      <c r="AH105" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -11012,9 +10514,6 @@
           <t>F3</t>
         </is>
       </c>
-      <c r="AH107" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -11041,9 +10540,6 @@
         <is>
           <t>F4</t>
         </is>
-      </c>
-      <c r="AH109" t="n">
-        <v>0.6</v>
       </c>
     </row>
   </sheetData>
@@ -12005,9 +11501,6 @@
           <t>D1</t>
         </is>
       </c>
-      <c r="AK55" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -12035,9 +11528,6 @@
           <t>D2</t>
         </is>
       </c>
-      <c r="AK57" t="n">
-        <v>10</v>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -12065,9 +11555,6 @@
           <t>D3</t>
         </is>
       </c>
-      <c r="AK59" t="n">
-        <v>14</v>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -12095,9 +11582,6 @@
           <t>D4</t>
         </is>
       </c>
-      <c r="AK61" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -12125,9 +11609,6 @@
           <t>D5</t>
         </is>
       </c>
-      <c r="AK63" t="n">
-        <v>10</v>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -12155,9 +11636,6 @@
           <t>D6</t>
         </is>
       </c>
-      <c r="AK65" t="n">
-        <v>12</v>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -12185,9 +11663,6 @@
           <t>D7</t>
         </is>
       </c>
-      <c r="AK67" t="n">
-        <v>22</v>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -12215,9 +11690,6 @@
           <t>D8</t>
         </is>
       </c>
-      <c r="AK69" t="n">
-        <v>20</v>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -12230,9 +11702,6 @@
           <t>E1</t>
         </is>
       </c>
-      <c r="AE70" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -12260,9 +11729,6 @@
           <t>E2</t>
         </is>
       </c>
-      <c r="AE72" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -12290,9 +11756,6 @@
           <t>E3</t>
         </is>
       </c>
-      <c r="AE74" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -12320,9 +11783,6 @@
           <t>E4</t>
         </is>
       </c>
-      <c r="AE76" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -12350,9 +11810,6 @@
           <t>E5</t>
         </is>
       </c>
-      <c r="AE78" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -12380,9 +11837,6 @@
           <t>E6</t>
         </is>
       </c>
-      <c r="AE80" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -12410,9 +11864,6 @@
           <t>E7</t>
         </is>
       </c>
-      <c r="AE82" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -12440,9 +11891,6 @@
           <t>E8</t>
         </is>
       </c>
-      <c r="AE84" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -12470,9 +11918,6 @@
           <t>E9</t>
         </is>
       </c>
-      <c r="AE86" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -12500,9 +11945,6 @@
           <t>E10</t>
         </is>
       </c>
-      <c r="AE88" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -12530,9 +11972,6 @@
           <t>E11</t>
         </is>
       </c>
-      <c r="AE90" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -12560,9 +11999,6 @@
           <t>E12</t>
         </is>
       </c>
-      <c r="AE92" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -12590,9 +12026,6 @@
           <t>E13</t>
         </is>
       </c>
-      <c r="AE94" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -12620,9 +12053,6 @@
           <t>E14</t>
         </is>
       </c>
-      <c r="AE96" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -12650,9 +12080,6 @@
           <t>E15</t>
         </is>
       </c>
-      <c r="AE98" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -12680,9 +12107,6 @@
           <t>E16</t>
         </is>
       </c>
-      <c r="AE100" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -12710,9 +12134,6 @@
           <t>F1</t>
         </is>
       </c>
-      <c r="AH102" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -12740,9 +12161,6 @@
           <t>F2</t>
         </is>
       </c>
-      <c r="AH104" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -12770,9 +12188,6 @@
           <t>F3</t>
         </is>
       </c>
-      <c r="AH106" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -12799,9 +12214,6 @@
         <is>
           <t>F4</t>
         </is>
-      </c>
-      <c r="AH108" t="n">
-        <v>0.6</v>
       </c>
     </row>
     <row r="109">

</xml_diff>